<commit_message>
parche el bug q duplica las lista en la vista listxlsx
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRAS 1842 DISMAY.xlsx
+++ b/LISTAS/ma/BISAGRAS 1842 DISMAY.xlsx
@@ -808,14 +808,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="22" t="n">
-        <v>45180.47732512275</v>
+        <v>45223</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -857,26 +853,6 @@
       <c r="A11" s="21" t="n"/>
       <c r="E11" s="7" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32" ht="18" customHeight="1" s="1">
       <c r="A32" s="24" t="inlineStr">
         <is>
@@ -908,7 +884,7 @@
       </c>
       <c r="C33" s="29" t="n"/>
       <c r="D33" s="30" t="n">
-        <v>105.52</v>
+        <v>116</v>
       </c>
       <c r="E33" s="31" t="n"/>
       <c r="F33" s="31" t="n"/>
@@ -927,7 +903,7 @@
       </c>
       <c r="C34" s="29" t="n"/>
       <c r="D34" s="32" t="n">
-        <v>116.342</v>
+        <v>126.813</v>
       </c>
       <c r="E34" s="31" t="n"/>
       <c r="F34" s="31" t="n"/>
@@ -946,7 +922,7 @@
       </c>
       <c r="C35" s="27" t="n"/>
       <c r="D35" s="32" t="n">
-        <v>137.283</v>
+        <v>149.638</v>
       </c>
       <c r="E35" s="31" t="n"/>
       <c r="F35" s="31" t="n"/>
@@ -1002,7 +978,7 @@
       </c>
       <c r="C39" s="29" t="n"/>
       <c r="D39" s="30" t="n">
-        <v>145.129</v>
+        <v>158.191</v>
       </c>
       <c r="E39" s="31" t="n"/>
       <c r="F39" s="31" t="n"/>
@@ -1021,7 +997,7 @@
       </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="32" t="n">
-        <v>223.133</v>
+        <v>243.215</v>
       </c>
       <c r="E40" s="31" t="n"/>
       <c r="F40" s="31" t="n"/>
@@ -1040,19 +1016,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="A37:D37"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A9:D9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>